<commit_message>
Add our offers count and average offer price to client RFQ file
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UTAIR_EXP_Frequent_RFQ.xlsx
+++ b/UTAIR_EXP_Frequent_RFQ.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Инструкция" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frequent RFQ'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frequent RFQ'!$A$1:$I$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,15 +32,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -92,10 +92,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -108,6 +108,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +126,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -490,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -548,7 +554,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RFQ count — number of separate requests (unique RFQs)</t>
+          <t>RFQ count — number of separate customer requests</t>
         </is>
       </c>
     </row>
@@ -562,19 +568,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Your purchase price EA (USD) — please enter your unit buy price</t>
+          <t>Our offers count — number of commercial offers we provided</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Currency note / comments — optional (e.g. MOQ, condition, validity)</t>
+          <t>Our average offer price EA (USD) — average unit price in our offers (DDP MOW basis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Your purchase price EA (USD) — please enter your unit buy price</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>Comments — optional (MOQ, condition, validity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Thank you!</t>
         </is>
@@ -591,19 +611,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>#</t>
@@ -631,12 +653,22 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>Our offers count</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Our average offer price EA (USD)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Your purchase price EA (USD)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Currency note / comments</t>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Comments</t>
         </is>
       </c>
     </row>
@@ -660,31 +692,43 @@
       <c r="E2" s="6" t="n">
         <v>67</v>
       </c>
-      <c r="F2" s="7" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr"/>
+      <c r="F2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>8560</v>
+      </c>
+      <c r="H2" s="8" t="inlineStr"/>
+      <c r="I2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
+      <c r="A3" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>810483-2</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>SEAL - CAP</t>
         </is>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
+      <c r="F3" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>5324</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr"/>
+      <c r="I3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -706,31 +750,43 @@
       <c r="E4" s="6" t="n">
         <v>288</v>
       </c>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
+      <c r="F4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="H4" s="8" t="inlineStr"/>
+      <c r="I4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="A5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>RAA2196-4</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>SWITCH</t>
         </is>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="11" t="n">
+      <c r="D5" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
+      <c r="F5" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>27933.33</v>
+      </c>
+      <c r="H5" s="8" t="inlineStr"/>
+      <c r="I5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -752,31 +808,43 @@
       <c r="E6" s="6" t="n">
         <v>1360</v>
       </c>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
+      <c r="F6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>149.33</v>
+      </c>
+      <c r="H6" s="8" t="inlineStr"/>
+      <c r="I6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>3036376</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>FILTER ELEMENT</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="11" t="n">
+      <c r="D7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="12" t="n">
         <v>48</v>
       </c>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="F7" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>1425.71</v>
+      </c>
+      <c r="H7" s="8" t="inlineStr"/>
+      <c r="I7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -798,31 +866,43 @@
       <c r="E8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
+      <c r="F8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>13433.33</v>
+      </c>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>67839</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>CARTRIDGE VALVE ASSY</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E9" s="11" t="n">
+      <c r="D9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
+      <c r="F9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>4803.33</v>
+      </c>
+      <c r="H9" s="8" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -844,31 +924,43 @@
       <c r="E10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
+      <c r="F10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>7583.33</v>
+      </c>
+      <c r="H10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>90G97</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>SWITCH</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="11" t="n">
+      <c r="D11" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
+      <c r="F11" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>11000</v>
+      </c>
+      <c r="H11" s="8" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -890,31 +982,43 @@
       <c r="E12" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
+      <c r="F12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>7005</v>
+      </c>
+      <c r="H12" s="8" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>141A6075-3</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>ARM ASSY</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="11" t="n">
+      <c r="D13" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
+      <c r="F13" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>13866.67</v>
+      </c>
+      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -936,31 +1040,43 @@
       <c r="E14" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="7" t="inlineStr"/>
+      <c r="F14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>4130</v>
+      </c>
+      <c r="H14" s="8" t="inlineStr"/>
+      <c r="I14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>038845-1</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>BRACKET-MOUNTING</t>
         </is>
       </c>
-      <c r="D15" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" s="11" t="n">
+      <c r="D15" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="7" t="inlineStr"/>
+      <c r="F15" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>1225</v>
+      </c>
+      <c r="H15" s="8" t="inlineStr"/>
+      <c r="I15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -982,31 +1098,43 @@
       <c r="E16" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="7" t="inlineStr"/>
+      <c r="F16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>670</v>
+      </c>
+      <c r="H16" s="8" t="inlineStr"/>
+      <c r="I16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="n">
+      <c r="A17" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>2100002-01-129</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>RESTRAINT SYSTEM - SYS</t>
         </is>
       </c>
-      <c r="D17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17" s="7" t="inlineStr"/>
-      <c r="G17" s="7" t="inlineStr"/>
+      <c r="D17" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>8266.67</v>
+      </c>
+      <c r="H17" s="8" t="inlineStr"/>
+      <c r="I17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1028,31 +1156,43 @@
       <c r="E18" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="7" t="inlineStr"/>
+      <c r="F18" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>1565</v>
+      </c>
+      <c r="H18" s="8" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="9" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>141A6076-1</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>PIN</t>
         </is>
       </c>
-      <c r="D19" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E19" s="11" t="n">
+      <c r="D19" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="F19" s="7" t="inlineStr"/>
-      <c r="G19" s="7" t="inlineStr"/>
+      <c r="F19" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>2035</v>
+      </c>
+      <c r="H19" s="8" t="inlineStr"/>
+      <c r="I19" s="8" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1074,31 +1214,43 @@
       <c r="E20" s="6" t="n">
         <v>105</v>
       </c>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="7" t="inlineStr"/>
+      <c r="F20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>295</v>
+      </c>
+      <c r="H20" s="8" t="inlineStr"/>
+      <c r="I20" s="8" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="n">
+      <c r="A21" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>65-90305-88</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>KIT - CFM56-7 FUEL PUMP FILTER</t>
         </is>
       </c>
-      <c r="D21" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" s="11" t="n">
+      <c r="D21" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="7" t="inlineStr"/>
+      <c r="F21" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="H21" s="8" t="inlineStr"/>
+      <c r="I21" s="8" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1120,31 +1272,43 @@
       <c r="E22" s="6" t="n">
         <v>690</v>
       </c>
-      <c r="F22" s="7" t="inlineStr"/>
-      <c r="G22" s="7" t="inlineStr"/>
+      <c r="F22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="H22" s="8" t="inlineStr"/>
+      <c r="I22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>65-90305-24</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>FILTER MAINTENANCE KIT</t>
         </is>
       </c>
-      <c r="D23" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E23" s="11" t="n">
+      <c r="D23" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="F23" s="7" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
+      <c r="F23" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>462.5</v>
+      </c>
+      <c r="H23" s="8" t="inlineStr"/>
+      <c r="I23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1166,31 +1330,43 @@
       <c r="E24" s="6" t="n">
         <v>3122</v>
       </c>
-      <c r="F24" s="7" t="inlineStr"/>
-      <c r="G24" s="7" t="inlineStr"/>
+      <c r="F24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>4.83</v>
+      </c>
+      <c r="H24" s="8" t="inlineStr"/>
+      <c r="I24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n">
+      <c r="A25" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>7577741</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>FILTER</t>
         </is>
       </c>
-      <c r="D25" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E25" s="11" t="n">
+      <c r="D25" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" s="12" t="n">
         <v>224</v>
       </c>
-      <c r="F25" s="7" t="inlineStr"/>
-      <c r="G25" s="7" t="inlineStr"/>
+      <c r="F25" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <v>48.25</v>
+      </c>
+      <c r="H25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1212,11 +1388,17 @@
       <c r="E26" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F26" s="7" t="inlineStr"/>
-      <c r="G26" s="7" t="inlineStr"/>
+      <c r="F26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>496.67</v>
+      </c>
+      <c r="H26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:I26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1227,7 +1409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1285,7 +1467,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RFQ count — число отдельных запросов</t>
+          <t>RFQ count — число отдельных запросов клиента</t>
         </is>
       </c>
     </row>
@@ -1299,19 +1481,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Your purchase price EA (USD) — ваша закупочная цена за единицу</t>
+          <t>Our offers count — сколько коммерческих предложений мы направили</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Comments — при необходимости (MOQ, состояние, срок действия цены)</t>
+          <t>Our average offer price EA (USD) — средняя цена за единицу в наших предложениях (база DDP MOW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Your purchase price EA (USD) — ваша закупочная цена за единицу</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>Comments — при необходимости (MOQ, состояние, срок действия цены)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Спасибо!</t>
         </is>

</xml_diff>

<commit_message>
Publish UTAIR_EXP_Frequent_RFQ_v2 with offers count and avg price columns
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UTAIR_EXP_Frequent_RFQ.xlsx
+++ b/UTAIR_EXP_Frequent_RFQ.xlsx
@@ -505,7 +505,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>UTAIR — Frequent expendable RFQs</t>
+          <t>UTAIR — Frequent expendable RFQs (v2)</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1418,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>UTAIR — Часто запрашиваемые расходные компоненты (EXP)</t>
+          <t>UTAIR — Часто запрашиваемые расходные компоненты (EXP) — v2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove thousand separators from qty column in client RFQ file
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UTAIR_EXP_Frequent_RFQ.xlsx
+++ b/UTAIR_EXP_Frequent_RFQ.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.##"/>
+    <numFmt numFmtId="165" formatCode="0.##"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -92,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,6 +130,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -497,7 +504,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
@@ -612,7 +619,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -689,7 +696,7 @@
       <c r="D2" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="6" t="n">
+      <c r="E2" s="14" t="n">
         <v>67</v>
       </c>
       <c r="F2" s="3" t="n">
@@ -718,7 +725,7 @@
       <c r="D3" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="E3" s="15" t="n">
         <v>18</v>
       </c>
       <c r="F3" s="9" t="n">
@@ -747,7 +754,7 @@
       <c r="D4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="14" t="n">
         <v>288</v>
       </c>
       <c r="F4" s="3" t="n">
@@ -776,7 +783,7 @@
       <c r="D5" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="15" t="n">
         <v>6</v>
       </c>
       <c r="F5" s="9" t="n">
@@ -805,7 +812,7 @@
       <c r="D6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="14" t="n">
         <v>1360</v>
       </c>
       <c r="F6" s="3" t="n">
@@ -834,7 +841,7 @@
       <c r="D7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="15" t="n">
         <v>48</v>
       </c>
       <c r="F7" s="9" t="n">
@@ -863,7 +870,7 @@
       <c r="D8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="14" t="n">
         <v>7</v>
       </c>
       <c r="F8" s="3" t="n">
@@ -892,7 +899,7 @@
       <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="15" t="n">
         <v>17</v>
       </c>
       <c r="F9" s="9" t="n">
@@ -921,7 +928,7 @@
       <c r="D10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="14" t="n">
         <v>9</v>
       </c>
       <c r="F10" s="3" t="n">
@@ -950,7 +957,7 @@
       <c r="D11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="15" t="n">
         <v>6</v>
       </c>
       <c r="F11" s="9" t="n">
@@ -979,7 +986,7 @@
       <c r="D12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="14" t="n">
         <v>25</v>
       </c>
       <c r="F12" s="3" t="n">
@@ -1008,7 +1015,7 @@
       <c r="D13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="15" t="n">
         <v>6</v>
       </c>
       <c r="F13" s="9" t="n">
@@ -1037,7 +1044,7 @@
       <c r="D14" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="14" t="n">
         <v>17</v>
       </c>
       <c r="F14" s="3" t="n">
@@ -1066,7 +1073,7 @@
       <c r="D15" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="15" t="n">
         <v>38</v>
       </c>
       <c r="F15" s="9" t="n">
@@ -1095,7 +1102,7 @@
       <c r="D16" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="6" t="n">
+      <c r="E16" s="14" t="n">
         <v>120</v>
       </c>
       <c r="F16" s="3" t="n">
@@ -1124,7 +1131,7 @@
       <c r="D17" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="15" t="n">
         <v>4</v>
       </c>
       <c r="F17" s="9" t="n">
@@ -1153,7 +1160,7 @@
       <c r="D18" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="6" t="n">
+      <c r="E18" s="14" t="n">
         <v>14</v>
       </c>
       <c r="F18" s="3" t="n">
@@ -1182,7 +1189,7 @@
       <c r="D19" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="15" t="n">
         <v>21</v>
       </c>
       <c r="F19" s="9" t="n">
@@ -1211,7 +1218,7 @@
       <c r="D20" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E20" s="6" t="n">
+      <c r="E20" s="14" t="n">
         <v>105</v>
       </c>
       <c r="F20" s="3" t="n">
@@ -1240,7 +1247,7 @@
       <c r="D21" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="15" t="n">
         <v>35</v>
       </c>
       <c r="F21" s="9" t="n">
@@ -1269,7 +1276,7 @@
       <c r="D22" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E22" s="6" t="n">
+      <c r="E22" s="14" t="n">
         <v>690</v>
       </c>
       <c r="F22" s="3" t="n">
@@ -1298,7 +1305,7 @@
       <c r="D23" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="12" t="n">
+      <c r="E23" s="15" t="n">
         <v>26</v>
       </c>
       <c r="F23" s="9" t="n">
@@ -1327,7 +1334,7 @@
       <c r="D24" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E24" s="6" t="n">
+      <c r="E24" s="14" t="n">
         <v>3122</v>
       </c>
       <c r="F24" s="3" t="n">
@@ -1356,7 +1363,7 @@
       <c r="D25" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="15" t="n">
         <v>224</v>
       </c>
       <c r="F25" s="9" t="n">
@@ -1385,7 +1392,7 @@
       <c r="D26" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E26" s="6" t="n">
+      <c r="E26" s="14" t="n">
         <v>20</v>
       </c>
       <c r="F26" s="3" t="n">
@@ -1410,7 +1417,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>

</xml_diff>

<commit_message>
Count 1 offer per ExpR including BOS; keep BOS out of average price only
Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UTAIR_EXP_Frequent_RFQ.xlsx
+++ b/UTAIR_EXP_Frequent_RFQ.xlsx
@@ -20,10 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0.##"/>
-    <numFmt numFmtId="165" formatCode="0.##"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -93,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -108,7 +105,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -126,16 +123,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -506,7 +497,7 @@
   <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -575,14 +566,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Our offers count — number of commercial offers we provided</t>
+          <t>Our offers count — number of commercial offers we sent (1 per RFQ; options calculated for comparison are not counted separately)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Our average offer price EA (USD) — average unit price in our offers (DDP MOW basis)</t>
+          <t>Our average offer price EA (USD) — average unit price of sent offers (DDP MOW basis)</t>
         </is>
       </c>
     </row>
@@ -696,7 +687,7 @@
       <c r="D2" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="6" t="n">
         <v>67</v>
       </c>
       <c r="F2" s="3" t="n">
@@ -725,7 +716,7 @@
       <c r="D3" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="12" t="n">
         <v>18</v>
       </c>
       <c r="F3" s="9" t="n">
@@ -754,7 +745,7 @@
       <c r="D4" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="6" t="n">
         <v>288</v>
       </c>
       <c r="F4" s="3" t="n">
@@ -783,7 +774,7 @@
       <c r="D5" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="12" t="n">
         <v>6</v>
       </c>
       <c r="F5" s="9" t="n">
@@ -812,7 +803,7 @@
       <c r="D6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="6" t="n">
         <v>1360</v>
       </c>
       <c r="F6" s="3" t="n">
@@ -841,14 +832,14 @@
       <c r="D7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="12" t="n">
         <v>48</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>1425.71</v>
+        <v>2146.67</v>
       </c>
       <c r="H7" s="8" t="inlineStr"/>
       <c r="I7" s="8" t="inlineStr"/>
@@ -870,7 +861,7 @@
       <c r="D8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="6" t="n">
         <v>7</v>
       </c>
       <c r="F8" s="3" t="n">
@@ -899,7 +890,7 @@
       <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="12" t="n">
         <v>17</v>
       </c>
       <c r="F9" s="9" t="n">
@@ -928,7 +919,7 @@
       <c r="D10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E10" s="6" t="n">
         <v>9</v>
       </c>
       <c r="F10" s="3" t="n">
@@ -957,7 +948,7 @@
       <c r="D11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="12" t="n">
         <v>6</v>
       </c>
       <c r="F11" s="9" t="n">
@@ -986,11 +977,11 @@
       <c r="D12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="6" t="n">
         <v>25</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>7005</v>
@@ -1015,7 +1006,7 @@
       <c r="D13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="12" t="n">
         <v>6</v>
       </c>
       <c r="F13" s="9" t="n">
@@ -1044,11 +1035,11 @@
       <c r="D14" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="6" t="n">
         <v>17</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>4130</v>
@@ -1073,7 +1064,7 @@
       <c r="D15" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="12" t="n">
         <v>38</v>
       </c>
       <c r="F15" s="9" t="n">
@@ -1102,7 +1093,7 @@
       <c r="D16" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="6" t="n">
         <v>120</v>
       </c>
       <c r="F16" s="3" t="n">
@@ -1131,7 +1122,7 @@
       <c r="D17" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="12" t="n">
         <v>4</v>
       </c>
       <c r="F17" s="9" t="n">
@@ -1160,7 +1151,7 @@
       <c r="D18" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="6" t="n">
         <v>14</v>
       </c>
       <c r="F18" s="3" t="n">
@@ -1189,7 +1180,7 @@
       <c r="D19" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="12" t="n">
         <v>21</v>
       </c>
       <c r="F19" s="9" t="n">
@@ -1218,11 +1209,11 @@
       <c r="D20" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="E20" s="6" t="n">
         <v>105</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>295</v>
@@ -1247,7 +1238,7 @@
       <c r="D21" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="12" t="n">
         <v>35</v>
       </c>
       <c r="F21" s="9" t="n">
@@ -1276,7 +1267,7 @@
       <c r="D22" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="6" t="n">
         <v>690</v>
       </c>
       <c r="F22" s="3" t="n">
@@ -1305,7 +1296,7 @@
       <c r="D23" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="15" t="n">
+      <c r="E23" s="12" t="n">
         <v>26</v>
       </c>
       <c r="F23" s="9" t="n">
@@ -1334,7 +1325,7 @@
       <c r="D24" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="E24" s="6" t="n">
         <v>3122</v>
       </c>
       <c r="F24" s="3" t="n">
@@ -1363,7 +1354,7 @@
       <c r="D25" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="15" t="n">
+      <c r="E25" s="12" t="n">
         <v>224</v>
       </c>
       <c r="F25" s="9" t="n">
@@ -1392,7 +1383,7 @@
       <c r="D26" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="E26" s="6" t="n">
         <v>20</v>
       </c>
       <c r="F26" s="3" t="n">
@@ -1419,7 +1410,7 @@
   <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1488,14 +1479,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Our offers count — сколько коммерческих предложений мы направили</t>
+          <t>Our offers count — число отправленных предложений (1 на RFQ; варианты «для сравнения» отдельно не считаются)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Our average offer price EA (USD) — средняя цена за единицу в наших предложениях (база DDP MOW)</t>
+          <t>Our average offer price EA (USD) — средняя цена за единицу в отправленных предложениях (база DDP MOW)</t>
         </is>
       </c>
     </row>

</xml_diff>